<commit_message>
Update project files and frontend fixes
</commit_message>
<xml_diff>
--- a/database_sheets/all_users.xlsx
+++ b/database_sheets/all_users.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -606,9 +606,32 @@
         <v>2026-07-08T13:17:20.915Z</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>mock_oxhnax576</v>
+      </c>
+      <c r="B10" t="str">
+        <v>joh</v>
+      </c>
+      <c r="C10" t="str">
+        <v>john@example.com</v>
+      </c>
+      <c r="D10" t="str">
+        <v>1234567890</v>
+      </c>
+      <c r="E10" t="str">
+        <v>21/10</v>
+      </c>
+      <c r="F10" t="str">
+        <v>customer</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-07-23T19:49:56.871Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>